<commit_message>
Actualizar libro con nuevos datos y regenerar HTMLs para GitHub Pages
Se han actualizado los datos y regenerado todos los HTMLs del libro de consultas de tendencias electorales.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/mapeo_partidos_matriz.xlsx
+++ b/data/mapeo_partidos_matriz.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://presidenciagobierno.sharepoint.com/sites/GPG_AnalisisyEstudio/Documentos compartidos/1_ELECCIONES GENERALES/Acumulación de encuestas/data/01_mapeo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://presidenciagobierno.sharepoint.com/sites/GPG_AnalisisyEstudio/Documentos compartidos/1_ELECCIONES GENERALES/Acumulacion de encuestas/data/01_mapeo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{82A932B5-4284-384E-95F2-60F877873CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{82A932B5-4284-384E-95F2-60F877873CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3513408A-E81D-4B41-9307-C3027998B408}"/>
   <bookViews>
-    <workbookView xWindow="5480" yWindow="5060" windowWidth="25640" windowHeight="14440" activeTab="1" xr2:uid="{ECCB56EF-59F4-8B4D-AFD5-5938926572D2}"/>
+    <workbookView xWindow="4380" yWindow="1620" windowWidth="25640" windowHeight="14440" activeTab="1" xr2:uid="{ECCB56EF-59F4-8B4D-AFD5-5938926572D2}"/>
   </bookViews>
   <sheets>
     <sheet name="recuerdo" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="162">
   <si>
     <t>recuerdo</t>
   </si>
@@ -484,6 +484,45 @@
   </si>
   <si>
     <t>Cs</t>
+  </si>
+  <si>
+    <t>Otros regionalistas</t>
+  </si>
+  <si>
+    <t>JxCAT-JUNTS</t>
+  </si>
+  <si>
+    <t>SALF / Se acabó la fiesta</t>
+  </si>
+  <si>
+    <t>Not asked</t>
+  </si>
+  <si>
+    <t>Aliança Catalana</t>
+  </si>
+  <si>
+    <t>No sabe todavía</t>
+  </si>
+  <si>
+    <t>Voto nulo</t>
+  </si>
+  <si>
+    <t>Se Acabó la Fiesta</t>
+  </si>
+  <si>
+    <t>PACMA</t>
+  </si>
+  <si>
+    <t>N.R.</t>
+  </si>
+  <si>
+    <t>No tenía derecho a voto</t>
+  </si>
+  <si>
+    <t>No tenía edad</t>
+  </si>
+  <si>
+    <t>CCa</t>
   </si>
 </sst>
 </file>
@@ -874,7 +913,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48AEF380-D529-9241-86CD-DA068B19B2F0}">
-  <dimension ref="A1:B110"/>
+  <dimension ref="A1:B117"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="78" bestFit="1" customWidth="1"/>
@@ -1761,6 +1800,62 @@
         <v>3</v>
       </c>
     </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>149</v>
+      </c>
+      <c r="B111" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>150</v>
+      </c>
+      <c r="B112" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>158</v>
+      </c>
+      <c r="B113" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>159</v>
+      </c>
+      <c r="B114" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>160</v>
+      </c>
+      <c r="B115" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>161</v>
+      </c>
+      <c r="B116" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>157</v>
+      </c>
+      <c r="B117" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1768,7 +1863,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7181B33D-8A70-444C-B0E7-DEF1CD502C3D}">
-  <dimension ref="A1:B110"/>
+  <dimension ref="A1:B119"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="94.83203125" bestFit="1" customWidth="1"/>
@@ -2654,14 +2749,97 @@
         <v>3</v>
       </c>
     </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>151</v>
+      </c>
+      <c r="B111" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>152</v>
+      </c>
+      <c r="B112" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>153</v>
+      </c>
+      <c r="B113" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>154</v>
+      </c>
+      <c r="B114" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>155</v>
+      </c>
+      <c r="B115" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>156</v>
+      </c>
+      <c r="B116" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>43</v>
+      </c>
+      <c r="B117" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>157</v>
+      </c>
+      <c r="B118" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>161</v>
+      </c>
+      <c r="B119" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100F5F30ABF65F76F448DBB03EC0DD2EDEB" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="94bd7b8a0020789c7b9989917fe587f8">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7516a298-e54c-4d8e-8268-8b2669e6c11c" xmlns:ns3="7500c241-b1f5-4397-96dd-287e9bb86023" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="41b27df312a9841dd5a5b07fdb90fe08" ns2:_="" ns3:_="">
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="7500c241-b1f5-4397-96dd-287e9bb86023" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7516a298-e54c-4d8e-8268-8b2669e6c11c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100F5F30ABF65F76F448DBB03EC0DD2EDEB" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="798453efef0eb178be7723a75e1e98a2">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7516a298-e54c-4d8e-8268-8b2669e6c11c" xmlns:ns3="7500c241-b1f5-4397-96dd-287e9bb86023" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="667ea7f6a5b01fa511919246a92461c2" ns2:_="" ns3:_="">
     <xsd:import namespace="7516a298-e54c-4d8e-8268-8b2669e6c11c"/>
     <xsd:import namespace="7500c241-b1f5-4397-96dd-287e9bb86023"/>
     <xsd:element name="properties">
@@ -2882,7 +3060,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2891,25 +3069,46 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="7500c241-b1f5-4397-96dd-287e9bb86023" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7516a298-e54c-4d8e-8268-8b2669e6c11c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79CCF8C3-86DD-42AD-B543-255DC050F7A6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CACCDEF-D398-4140-8C23-5DA56778A26C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="7516a298-e54c-4d8e-8268-8b2669e6c11c"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="7500c241-b1f5-4397-96dd-287e9bb86023"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2308DF1-1179-4B09-8F46-879FC5A8821D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C83BB5EA-0AD3-473D-AF2D-C4F591FA1545}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="7516a298-e54c-4d8e-8268-8b2669e6c11c"/>
+    <ds:schemaRef ds:uri="7500c241-b1f5-4397-96dd-287e9bb86023"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CACCDEF-D398-4140-8C23-5DA56778A26C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2308DF1-1179-4B09-8F46-879FC5A8821D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>